<commit_message>
accessibilité : correction des 7 non-conformités RGAA relevées
- 6.1 : les noms accessibles commencent par l'intitulé visible
  (« Prendre RDV », « Plaquette PDF · 6 pages », « Télécharger le PDF »).
- 3.3 : bordure des champs et des puces du formulaire en --ink-quiet
  (1,51:1 → 5,57:1, seuil 3:1).
- 10.6 : liens soulignés dans l'adresse de contact et les lignes des
  mentions légales (dd a).
- 8.2 : identifiant « jouons-ensemble » en double sur /projets/ (la carte
  devient « projet-jouons-ensemble »).
- 8.9 : <i> remplacé par <span> dans la légende de CommuneMap.
- 10.11 : la plaquette devient fluide à l'écran sous 760 px (grilles sur
  une colonne) ; l'A4 reste à l'impression, PDF régénéré (6 pages).
- 12.7 : lien « Aller au contenu » sur la plaquette.

Grille d'audit mise à jour : 48 C, 0 NC, 43 NA, 15 à tester à la main.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/audit-rgaa/grille-audit-rgaa-pxlc.xlsx
+++ b/docs/audit-rgaa/grille-audit-rgaa-pxlc.xlsx
@@ -555,7 +555,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Pré-remplie le 21/09/2026 à partir du build du site (tests automatisés jsdom, axe-core, Playwright, calculs de contraste) et de la lecture du code.</t>
+          <t>Pré-remplie le 21/09/2026 à partir du build du site (tests automatisés jsdom, axe-core, Playwright, calculs de contraste) et de la lecture du code. Les 7 non-conformités relevées ont été corrigées le même jour (onglet « Corrections »).</t>
         </is>
       </c>
     </row>
@@ -2190,7 +2190,7 @@
       </c>
       <c r="G15" s="14" t="inlineStr">
         <is>
-          <t>NC</t>
+          <t>C</t>
         </is>
       </c>
       <c r="H15" s="14" t="inlineStr">
@@ -2214,7 +2214,7 @@
       </c>
       <c r="L15" s="12" t="inlineStr">
         <is>
-          <t>Contact : bordure des champs et des puces de choix = --line, 1,51:1 contre le fond du champ (seuil 3:1). Ailleurs, les boutons à bordure (thème, menu) sont identifiables par leur icône, contrastée.</t>
+          <t>Corrigé le 21/09/2026 : bordure des champs et des puces de choix en --ink-quiet (5,57:1 sur blanc en clair, 4,75:1 en sombre ; seuil 3:1). Les boutons à bordure (thème, menu) sont identifiables par leur icône, contrastée.</t>
         </is>
       </c>
       <c r="M15" s="16" t="n"/>
@@ -3649,37 +3649,37 @@
       </c>
       <c r="D37" s="14" t="inlineStr">
         <is>
-          <t>NC</t>
+          <t>C</t>
         </is>
       </c>
       <c r="E37" s="14" t="inlineStr">
         <is>
-          <t>NC</t>
+          <t>C</t>
         </is>
       </c>
       <c r="F37" s="14" t="inlineStr">
         <is>
-          <t>NC</t>
+          <t>C</t>
         </is>
       </c>
       <c r="G37" s="14" t="inlineStr">
         <is>
-          <t>NC</t>
+          <t>C</t>
         </is>
       </c>
       <c r="H37" s="14" t="inlineStr">
         <is>
-          <t>NC</t>
+          <t>C</t>
         </is>
       </c>
       <c r="I37" s="14" t="inlineStr">
         <is>
-          <t>NC</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J37" s="14" t="inlineStr">
         <is>
-          <t>NC</t>
+          <t>C</t>
         </is>
       </c>
       <c r="K37" s="15">
@@ -3688,7 +3688,7 @@
       </c>
       <c r="L37" s="12" t="inlineStr">
         <is>
-          <t>Nom accessible ≠ intitulé visible (critère 6.1, test 6.1.5) : bouton d'en-tête visible « Prendre RDV » mais aria-label « Prendre rendez-vous (nouvel onglet) » (toutes les pages du site) ; À propos et Projets : « Plaquette PDF · 6 pages » → aria-label « Plaquette PDF, 6 pages… » ; Plaquette : « Télécharger le PDF » → « Télécharger la plaquette… ».</t>
+          <t>Corrigé le 21/09/2026 : chaque nom accessible commence par l'intitulé visible (« Prendre RDV (rendez-vous, nouvel onglet) », « Plaquette PDF · 6 pages (nouvel onglet) », « Télécharger le PDF (plaquette, 6 pages, nouvel onglet) »). Contrôle automatisé sur toutes les pages : 0 écart. Liens contextuels (« Voir le projet ») explicites par leur contexte.</t>
         </is>
       </c>
       <c r="M37" s="16" t="n"/>
@@ -4195,7 +4195,7 @@
       </c>
       <c r="F45" s="14" t="inlineStr">
         <is>
-          <t>NC</t>
+          <t>AT</t>
         </is>
       </c>
       <c r="G45" s="14" t="inlineStr">
@@ -4224,7 +4224,7 @@
       </c>
       <c r="L45" s="12" t="inlineStr">
         <is>
-          <t>Projets : identifiant « jouons-ensemble » en double (carte projet + section). Autres pages : passer le validateur W3C.</t>
+          <t>Identifiant dupliqué de Projets corrigé le 21/09/2026 (carte renommée « projet-jouons-ensemble ») ; plus aucun id en double sur l'échantillon. Reste à passer le validateur W3C sur chaque page.</t>
         </is>
       </c>
       <c r="M45" s="16" t="n"/>
@@ -4669,7 +4669,7 @@
       </c>
       <c r="G52" s="14" t="inlineStr">
         <is>
-          <t>NC</t>
+          <t>C</t>
         </is>
       </c>
       <c r="H52" s="14" t="inlineStr">
@@ -4693,7 +4693,7 @@
       </c>
       <c r="L52" s="12" t="inlineStr">
         <is>
-          <t>Contact : balise &lt;i&gt; utilisée pour styliser les numéros de la légende de la carte (présentation seule).</t>
+          <t>Corrigé le 21/09/2026 : les numéros de la légende de la carte (contact) passent de &lt;i&gt; à &lt;span&gt;. Aucune autre balise utilisée pour la seule présentation.</t>
         </is>
       </c>
       <c r="M52" s="16" t="n"/>
@@ -5287,7 +5287,7 @@
       </c>
       <c r="J61" s="14" t="inlineStr">
         <is>
-          <t>AT</t>
+          <t>C</t>
         </is>
       </c>
       <c r="K61" s="15">
@@ -5296,7 +5296,7 @@
       </c>
       <c r="L61" s="12" t="inlineStr">
         <is>
-          <t>Pages du site : aucun débordement à 320 px de large (équivalent d'un zoom 400 % sur 1280 px). Plaquette : feuilles A4 de largeur fixe, vérifier à 200 %.</t>
+          <t>Aucun débordement ni texte coupé à 320 px de large (équivalent d'un zoom 400 % sur 1280 px), plaquette comprise depuis le 21/09/2026 (feuilles fluides sous 760 px).</t>
         </is>
       </c>
       <c r="M61" s="16" t="n"/>
@@ -5406,12 +5406,12 @@
       </c>
       <c r="G63" s="14" t="inlineStr">
         <is>
-          <t>NC</t>
+          <t>C</t>
         </is>
       </c>
       <c r="H63" s="14" t="inlineStr">
         <is>
-          <t>NC</t>
+          <t>C</t>
         </is>
       </c>
       <c r="I63" s="14" t="inlineStr">
@@ -5430,7 +5430,7 @@
       </c>
       <c r="L63" s="12" t="inlineStr">
         <is>
-          <t>Liens sans soulignement dans du texte : contact (téléphone, email de l'adresse) et mentions légales (liens des lignes Téléphone, Email, LinkedIn). Couleur lien/texte = 1,64:1 en clair, 1,07:1 en sombre (seuil 3:1).</t>
+          <t>Corrigé le 21/09/2026 : liens soulignés dans l'adresse de contact et dans les lignes des mentions légales (la couleur seule, 1,64:1, ne suffisait pas). Liens de paragraphes et de listes déjà soulignés.</t>
         </is>
       </c>
       <c r="M63" s="16" t="n"/>
@@ -5756,7 +5756,7 @@
       </c>
       <c r="J68" s="14" t="inlineStr">
         <is>
-          <t>NC</t>
+          <t>C</t>
         </is>
       </c>
       <c r="K68" s="15">
@@ -5765,7 +5765,7 @@
       </c>
       <c r="L68" s="12" t="inlineStr">
         <is>
-          <t>Pages du site : aucun défilement horizontal à 320 px de large ni à 256 px de haut (corrigé le 21/09 : liens légaux du pied de page). Plaquette : feuilles A4 fixes, 237 px de débordement à 320 px.</t>
+          <t>Aucun défilement horizontal à 320 px de large ni à 256 px de haut sur les 7 pages (corrigé le 21/09/2026 : liens légaux du pied de page ; plaquette fluide à l'écran sous 760 px, A4 conservé à l'impression).</t>
         </is>
       </c>
       <c r="M68" s="16" t="n"/>
@@ -7297,7 +7297,7 @@
       </c>
       <c r="J91" s="14" t="inlineStr">
         <is>
-          <t>NC</t>
+          <t>C</t>
         </is>
       </c>
       <c r="K91" s="15">
@@ -7306,7 +7306,7 @@
       </c>
       <c r="L91" s="12" t="inlineStr">
         <is>
-          <t>Lien « Aller au contenu » → #main sur les pages du site. Plaquette : pas de lien d'évitement.</t>
+          <t>Lien « Aller au contenu » → #main sur les 7 pages (ajouté à la plaquette le 21/09/2026).</t>
         </is>
       </c>
       <c r="M91" s="16" t="n"/>
@@ -8527,7 +8527,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E8"/>
+  <dimension ref="A1:F8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -8535,6 +8535,7 @@
     <col width="55" customWidth="1" min="3" max="3"/>
     <col width="70" customWidth="1" min="4" max="4"/>
     <col width="9" customWidth="1" min="5" max="5"/>
+    <col width="20" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -8555,12 +8556,17 @@
       </c>
       <c r="D1" s="9" t="inlineStr">
         <is>
-          <t>Correction proposée</t>
+          <t>Correction</t>
         </is>
       </c>
       <c r="E1" s="9" t="inlineStr">
         <is>
           <t>Effort</t>
+        </is>
+      </c>
+      <c r="F1" s="9" t="inlineStr">
+        <is>
+          <t>État</t>
         </is>
       </c>
     </row>
@@ -8590,6 +8596,11 @@
           <t>Faible</t>
         </is>
       </c>
+      <c r="F2" s="12" t="inlineStr">
+        <is>
+          <t>Corrigé le 21/09/2026</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="12" t="inlineStr">
@@ -8617,6 +8628,11 @@
           <t>Faible</t>
         </is>
       </c>
+      <c r="F3" s="12" t="inlineStr">
+        <is>
+          <t>Corrigé le 21/09/2026</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="12" t="inlineStr">
@@ -8644,6 +8660,11 @@
           <t>Faible</t>
         </is>
       </c>
+      <c r="F4" s="12" t="inlineStr">
+        <is>
+          <t>Corrigé le 21/09/2026</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="12" t="inlineStr">
@@ -8671,6 +8692,11 @@
           <t>Faible</t>
         </is>
       </c>
+      <c r="F5" s="12" t="inlineStr">
+        <is>
+          <t>Corrigé le 21/09/2026</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="12" t="inlineStr">
@@ -8698,6 +8724,11 @@
           <t>Faible</t>
         </is>
       </c>
+      <c r="F6" s="12" t="inlineStr">
+        <is>
+          <t>Corrigé le 21/09/2026</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="12" t="inlineStr">
@@ -8725,6 +8756,11 @@
           <t>Moyen</t>
         </is>
       </c>
+      <c r="F7" s="12" t="inlineStr">
+        <is>
+          <t>Corrigé le 21/09/2026</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="12" t="inlineStr">
@@ -8750,6 +8786,11 @@
       <c r="E8" s="12" t="inlineStr">
         <is>
           <t>Faible</t>
+        </is>
+      </c>
+      <c r="F8" s="12" t="inlineStr">
+        <is>
+          <t>Corrigé le 21/09/2026</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
plaquette : lien vers la version web à côté de chaque lien PDF
« Lire en ligne » (héros de l'accueil, d'À propos et de Projets, menu
mobile) et « Lire la plaquette en ligne » (pied de page) mènent à
/plaquette/, version HTML dont le PDF est imprimé : le document
téléchargeable a sa version accessible (RGAA 13.3 et 13.4, conformes).
HeroSection accepte un lien texte ctaSecondaryAlt à côté du CTA
secondaire.

Grille d'audit : 50 C, 0 NC, 43 NA, 13 à tester.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/audit-rgaa/grille-audit-rgaa-pxlc.xlsx
+++ b/docs/audit-rgaa/grille-audit-rgaa-pxlc.xlsx
@@ -7736,37 +7736,37 @@
       </c>
       <c r="D98" s="14" t="inlineStr">
         <is>
-          <t>AT</t>
+          <t>C</t>
         </is>
       </c>
       <c r="E98" s="14" t="inlineStr">
         <is>
-          <t>AT</t>
+          <t>C</t>
         </is>
       </c>
       <c r="F98" s="14" t="inlineStr">
         <is>
-          <t>AT</t>
+          <t>C</t>
         </is>
       </c>
       <c r="G98" s="14" t="inlineStr">
         <is>
-          <t>AT</t>
+          <t>C</t>
         </is>
       </c>
       <c r="H98" s="14" t="inlineStr">
         <is>
-          <t>AT</t>
+          <t>C</t>
         </is>
       </c>
       <c r="I98" s="14" t="inlineStr">
         <is>
-          <t>AT</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J98" s="14" t="inlineStr">
         <is>
-          <t>AT</t>
+          <t>C</t>
         </is>
       </c>
       <c r="K98" s="15">
@@ -7775,7 +7775,7 @@
       </c>
       <c r="L98" s="12" t="inlineStr">
         <is>
-          <t>Plaquette PDF liée depuis toutes les pages. Soit vérifier que le PDF est balisé (PAC 2024), soit proposer la version HTML (/plaquette/) à côté de chaque lien PDF.</t>
+          <t>Depuis le 21/09/2026, chaque lien vers la plaquette PDF (héros, pied de page, menu mobile, déclaration) est accompagné d'un lien « Lire en ligne » / « Lire la plaquette en ligne » vers sa version HTML accessible (/plaquette/). Contrôle automatisé : autant de liens web que de liens PDF sur chaque page.</t>
         </is>
       </c>
       <c r="M98" s="16" t="n"/>
@@ -7803,37 +7803,37 @@
       </c>
       <c r="D99" s="14" t="inlineStr">
         <is>
-          <t>AT</t>
+          <t>C</t>
         </is>
       </c>
       <c r="E99" s="14" t="inlineStr">
         <is>
-          <t>AT</t>
+          <t>C</t>
         </is>
       </c>
       <c r="F99" s="14" t="inlineStr">
         <is>
-          <t>AT</t>
+          <t>C</t>
         </is>
       </c>
       <c r="G99" s="14" t="inlineStr">
         <is>
-          <t>AT</t>
+          <t>C</t>
         </is>
       </c>
       <c r="H99" s="14" t="inlineStr">
         <is>
-          <t>AT</t>
+          <t>C</t>
         </is>
       </c>
       <c r="I99" s="14" t="inlineStr">
         <is>
-          <t>AT</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J99" s="14" t="inlineStr">
         <is>
-          <t>AT</t>
+          <t>C</t>
         </is>
       </c>
       <c r="K99" s="15">
@@ -7842,7 +7842,7 @@
       </c>
       <c r="L99" s="12" t="inlineStr">
         <is>
-          <t>La page /plaquette/ est la source du PDF (même contenu) — conforme dès que 13.3 la propose comme version accessible.</t>
+          <t>La page /plaquette/ est la source dont le PDF est imprimé : même information, même structure.</t>
         </is>
       </c>
       <c r="M99" s="16" t="n"/>
@@ -8527,7 +8527,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F8"/>
+  <dimension ref="A1:F9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -8794,6 +8794,38 @@
         </is>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" s="12" t="inlineStr">
+        <is>
+          <t>13.3</t>
+        </is>
+      </c>
+      <c r="B9" s="12" t="inlineStr">
+        <is>
+          <t>Toutes</t>
+        </is>
+      </c>
+      <c r="C9" s="12" t="inlineStr">
+        <is>
+          <t>Plaquette PDF sans version accessible proposée à côté du lien (critère alors à tester).</t>
+        </is>
+      </c>
+      <c r="D9" s="12" t="inlineStr">
+        <is>
+          <t>Lien « Lire en ligne » vers /plaquette/ à côté de chaque lien PDF.</t>
+        </is>
+      </c>
+      <c r="E9" s="12" t="inlineStr">
+        <is>
+          <t>Faible</t>
+        </is>
+      </c>
+      <c r="F9" s="12" t="inlineStr">
+        <is>
+          <t>Corrigé le 21/09/2026</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -8805,7 +8837,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E14"/>
+  <dimension ref="A1:E13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -9088,106 +9120,79 @@
     <row r="11">
       <c r="A11" s="12" t="inlineStr">
         <is>
-          <t>13.3 · 13.4</t>
+          <t>13.5 · 13.6</t>
         </is>
       </c>
       <c r="B11" s="12" t="inlineStr">
         <is>
-          <t>Toutes</t>
+          <t>Plaquette (HTML)</t>
         </is>
       </c>
       <c r="C11" s="12" t="inlineStr">
         <is>
-          <t>PAC 2024 (gratuit, pdfua.foundation) ou Acrobat « Vérifier l'accessibilité »</t>
+          <t>NVDA</t>
         </is>
       </c>
       <c r="D11" s="12" t="inlineStr">
         <is>
-          <t>Ouvrir plaquette-pxlc.pdf dans PAC. Ou décider de proposer la version HTML /plaquette/ à côté de chaque lien PDF.</t>
+          <t>Écouter le coupon de consentement (« Fait à ........ le ...... »).</t>
         </is>
       </c>
       <c r="E11" s="12" t="inlineStr">
         <is>
-          <t>PDF balisé sans erreur PDF/UA bloquante, OU lien vers la version HTML à côté de chaque lien PDF.</t>
+          <t>Les pointillés ne sont pas lus caractère par caractère (sinon : les masquer aux lecteurs d'écran et donner une consigne textuelle).</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="12" t="inlineStr">
         <is>
-          <t>13.5 · 13.6</t>
+          <t>3.1</t>
         </is>
       </c>
       <c r="B12" s="12" t="inlineStr">
         <is>
-          <t>Plaquette (HTML)</t>
+          <t>Contact</t>
         </is>
       </c>
       <c r="C12" s="12" t="inlineStr">
         <is>
-          <t>NVDA</t>
+          <t>Œil + niveaux de gris (extension ou impression N&amp;B)</t>
         </is>
       </c>
       <c r="D12" s="12" t="inlineStr">
         <is>
-          <t>Écouter le coupon de consentement (« Fait à ........ le ...... »).</t>
+          <t>Regarder la carte des communes en niveaux de gris.</t>
         </is>
       </c>
       <c r="E12" s="12" t="inlineStr">
         <is>
-          <t>Les pointillés ne sont pas lus caractère par caractère (sinon : les masquer aux lecteurs d'écran et donner une consigne textuelle).</t>
+          <t>Les communes de la zone restent identifiables (numéros, légende) sans la couleur.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="12" t="inlineStr">
         <is>
-          <t>3.1</t>
+          <t>12.9</t>
         </is>
       </c>
       <c r="B13" s="12" t="inlineStr">
         <is>
-          <t>Contact</t>
+          <t>Toutes</t>
         </is>
       </c>
       <c r="C13" s="12" t="inlineStr">
         <is>
-          <t>Œil + niveaux de gris (extension ou impression N&amp;B)</t>
+          <t>Clavier, fenêtre &lt; 1024 px</t>
         </is>
       </c>
       <c r="D13" s="12" t="inlineStr">
         <is>
-          <t>Regarder la carte des communes en niveaux de gris.</t>
+          <t>Ouvrir le menu mobile au clavier, Tab plusieurs fois, puis Échap.</t>
         </is>
       </c>
       <c r="E13" s="12" t="inlineStr">
-        <is>
-          <t>Les communes de la zone restent identifiables (numéros, légende) sans la couleur.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="12" t="inlineStr">
-        <is>
-          <t>12.9</t>
-        </is>
-      </c>
-      <c r="B14" s="12" t="inlineStr">
-        <is>
-          <t>Toutes</t>
-        </is>
-      </c>
-      <c r="C14" s="12" t="inlineStr">
-        <is>
-          <t>Clavier, fenêtre &lt; 1024 px</t>
-        </is>
-      </c>
-      <c r="D14" s="12" t="inlineStr">
-        <is>
-          <t>Ouvrir le menu mobile au clavier, Tab plusieurs fois, puis Échap.</t>
-        </is>
-      </c>
-      <c r="E14" s="12" t="inlineStr">
         <is>
           <t>Le focus reste dans le menu tant qu'il est ouvert ; Échap le ferme et rend le focus.</t>
         </is>

</xml_diff>

<commit_message>
a11y : tests RGAA manuels, trois corrections
- 9.3 : repères chiffrés de l'accueil balisés en ul/li
- 10.12 : feuilles de la plaquette HTML en hauteur minimale A4 à l'écran,
  le texte n'est plus rogné quand l'espacement augmente (impression et
  PDF inchangés)
- 8.7 : anglicismes francisés (Devise du projet, Animateur de
  communauté, alternatives d'images sans « gaming »)

Grille d'audit mise à jour : 8.2, 9.1, 3.1, 10.2, 10.3 conformes ;
restent les 5 critères à tester au lecteur d'écran.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/audit-rgaa/grille-audit-rgaa-pxlc.xlsx
+++ b/docs/audit-rgaa/grille-audit-rgaa-pxlc.xlsx
@@ -555,7 +555,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Pré-remplie le 21/09/2026 à partir du build du site (tests automatisés jsdom, axe-core, Playwright, calculs de contraste) et de la lecture du code. Les 7 non-conformités relevées ont été corrigées le même jour (onglet « Corrections »).</t>
+          <t>Pré-remplie le 21/09/2026 à partir du build du site (tests automatisés jsdom, axe-core, Playwright, calculs de contraste) et de la lecture du code. Les 7 non-conformités relevées ont été corrigées le même jour (onglet « Corrections »). Mise à jour le 22/09/2026 : validateur W3C passé, tests 3.1, 8.7, 9.1, 9.3, 10.2, 10.3 et 10.12 faits (3 nouvelles corrections). Restent les tests au lecteur d'écran (NVDA).</t>
         </is>
       </c>
     </row>
@@ -2056,7 +2056,7 @@
       </c>
       <c r="G13" s="14" t="inlineStr">
         <is>
-          <t>AT</t>
+          <t>C</t>
         </is>
       </c>
       <c r="H13" s="14" t="inlineStr">
@@ -2083,7 +2083,11 @@
           <t>Lien actif du menu : couleur + barre + aria-current="page". Champs requis : astérisque + légende « Champs requis ». Contact : vérifier que la carte distingue la zone autrement que par la couleur (numéros).</t>
         </is>
       </c>
-      <c r="M13" s="16" t="n"/>
+      <c r="M13" s="16" t="inlineStr">
+        <is>
+          <t>22/09/2026 — Carte des communes en niveaux de gris : les 4 communes de la zone restent identifiables par leurs pastilles numérotées et la légende textuelle.</t>
+        </is>
+      </c>
       <c r="N13" s="17" t="inlineStr">
         <is>
           <t>Critère 3.1</t>
@@ -4185,37 +4189,37 @@
       </c>
       <c r="D45" s="14" t="inlineStr">
         <is>
-          <t>AT</t>
+          <t>C</t>
         </is>
       </c>
       <c r="E45" s="14" t="inlineStr">
         <is>
-          <t>AT</t>
+          <t>C</t>
         </is>
       </c>
       <c r="F45" s="14" t="inlineStr">
         <is>
-          <t>AT</t>
+          <t>C</t>
         </is>
       </c>
       <c r="G45" s="14" t="inlineStr">
         <is>
-          <t>AT</t>
+          <t>C</t>
         </is>
       </c>
       <c r="H45" s="14" t="inlineStr">
         <is>
-          <t>AT</t>
+          <t>C</t>
         </is>
       </c>
       <c r="I45" s="14" t="inlineStr">
         <is>
-          <t>AT</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J45" s="14" t="inlineStr">
         <is>
-          <t>AT</t>
+          <t>C</t>
         </is>
       </c>
       <c r="K45" s="15">
@@ -4227,7 +4231,11 @@
           <t>Identifiant dupliqué de Projets corrigé le 21/09/2026 (carte renommée « projet-jouons-ensemble ») ; plus aucun id en double sur l'échantillon. Reste à passer le validateur W3C sur chaque page.</t>
         </is>
       </c>
-      <c r="M45" s="16" t="n"/>
+      <c r="M45" s="16" t="inlineStr">
+        <is>
+          <t>22/09/2026 — Nu Html Checker (validator.w3.org, vnu 26.9.16) sur les 7 pages : 0 erreur. Avertissements « info » seulement : role="list" voulu (VoiceOver), alerte CSP des &lt;style&gt; inline = faux positif (hashes présents dans style-src). aria-required redondant retiré (PR #292).</t>
+        </is>
+      </c>
       <c r="N45" s="17" t="inlineStr">
         <is>
           <t>Critère 8.2</t>
@@ -4520,37 +4528,37 @@
       </c>
       <c r="D50" s="14" t="inlineStr">
         <is>
-          <t>AT</t>
+          <t>C</t>
         </is>
       </c>
       <c r="E50" s="14" t="inlineStr">
         <is>
-          <t>AT</t>
+          <t>C</t>
         </is>
       </c>
       <c r="F50" s="14" t="inlineStr">
         <is>
-          <t>AT</t>
+          <t>C</t>
         </is>
       </c>
       <c r="G50" s="14" t="inlineStr">
         <is>
-          <t>AT</t>
+          <t>C</t>
         </is>
       </c>
       <c r="H50" s="14" t="inlineStr">
         <is>
-          <t>AT</t>
+          <t>C</t>
         </is>
       </c>
       <c r="I50" s="14" t="inlineStr">
         <is>
-          <t>AT</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J50" s="14" t="inlineStr">
         <is>
-          <t>AT</t>
+          <t>C</t>
         </is>
       </c>
       <c r="K50" s="15">
@@ -4562,7 +4570,11 @@
           <t>Aucun changement de langue déclaré. Vérifier les mots anglais non passés dans l'usage (« gaming », « Duo gaming ») ; les noms propres (Destreland Gaming Cup) sont exemptés.</t>
         </is>
       </c>
-      <c r="M50" s="16" t="n"/>
+      <c r="M50" s="16" t="inlineStr">
+        <is>
+          <t>22/09/2026 — Relevé des mots étrangers : noms propres exemptés (Destreland Gaming Cup, Game Over Challenge, Atlantica Online, LinkedIn) ; esport, email, design dans l'usage. Francisés : « Tagline » → « Devise », « Community Manager » → « Animateur de communauté », « gaming » retiré de 2 alternatives d'images.</t>
+        </is>
+      </c>
       <c r="N50" s="17" t="inlineStr">
         <is>
           <t>Critère 8.7</t>
@@ -4788,7 +4800,7 @@
       </c>
       <c r="D54" s="14" t="inlineStr">
         <is>
-          <t>AT</t>
+          <t>C</t>
         </is>
       </c>
       <c r="E54" s="14" t="inlineStr">
@@ -4830,7 +4842,11 @@
           <t>Hiérarchie h1→h2→h3 cohérente. Accueil : « Quelques repères » et « Partenaires de confiance » ont l'apparence d'intitulés de section sans être des titres hx — à arbitrer.</t>
         </is>
       </c>
-      <c r="M54" s="16" t="n"/>
+      <c r="M54" s="16" t="inlineStr">
+        <is>
+          <t>22/09/2026 — « Quelques repères » balisé en h2 (PR #288) ; « Partenaires de confiance » est le libellé de la section PartnerStrip, nommée par aria-label.</t>
+        </is>
+      </c>
       <c r="N54" s="17" t="inlineStr">
         <is>
           <t>Critère 9.1</t>
@@ -4922,7 +4938,7 @@
       </c>
       <c r="D56" s="14" t="inlineStr">
         <is>
-          <t>AT</t>
+          <t>C</t>
         </is>
       </c>
       <c r="E56" s="14" t="inlineStr">
@@ -4964,7 +4980,11 @@
           <t>Listes balisées (ul/ol/dl). Accueil : vérifier la grille des 4 repères chiffrés, visuellement une liste mais balisée en div.</t>
         </is>
       </c>
-      <c r="M56" s="16" t="n"/>
+      <c r="M56" s="16" t="inlineStr">
+        <is>
+          <t>22/09/2026 — Les 4 repères chiffrés de l'accueil passent de div en ul/li (liste non ordonnée).</t>
+        </is>
+      </c>
       <c r="N56" s="17" t="inlineStr">
         <is>
           <t>Critère 9.3</t>
@@ -5123,37 +5143,37 @@
       </c>
       <c r="D59" s="14" t="inlineStr">
         <is>
-          <t>AT</t>
+          <t>C</t>
         </is>
       </c>
       <c r="E59" s="14" t="inlineStr">
         <is>
-          <t>AT</t>
+          <t>C</t>
         </is>
       </c>
       <c r="F59" s="14" t="inlineStr">
         <is>
-          <t>AT</t>
+          <t>C</t>
         </is>
       </c>
       <c r="G59" s="14" t="inlineStr">
         <is>
-          <t>AT</t>
+          <t>C</t>
         </is>
       </c>
       <c r="H59" s="14" t="inlineStr">
         <is>
-          <t>AT</t>
+          <t>C</t>
         </is>
       </c>
       <c r="I59" s="14" t="inlineStr">
         <is>
-          <t>AT</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J59" s="14" t="inlineStr">
         <is>
-          <t>AT</t>
+          <t>C</t>
         </is>
       </c>
       <c r="K59" s="15">
@@ -5165,7 +5185,11 @@
           <t>Désactiver les styles et vérifier que rien de porteur d'information ne disparaît (flèches → et points corail sont décoratifs).</t>
         </is>
       </c>
-      <c r="M59" s="16" t="n"/>
+      <c r="M59" s="16" t="inlineStr">
+        <is>
+          <t>22/09/2026 — Feuilles de style désactivées sur les 7 pages : tout le texte porteur d'information reste présent (contenus CSS générés = flèches, point, séparateurs, +/− de FAQ, tous décoratifs).</t>
+        </is>
+      </c>
       <c r="N59" s="17" t="inlineStr">
         <is>
           <t>Critère 10.2</t>
@@ -5190,37 +5214,37 @@
       </c>
       <c r="D60" s="14" t="inlineStr">
         <is>
-          <t>AT</t>
+          <t>C</t>
         </is>
       </c>
       <c r="E60" s="14" t="inlineStr">
         <is>
-          <t>AT</t>
+          <t>C</t>
         </is>
       </c>
       <c r="F60" s="14" t="inlineStr">
         <is>
-          <t>AT</t>
+          <t>C</t>
         </is>
       </c>
       <c r="G60" s="14" t="inlineStr">
         <is>
-          <t>AT</t>
+          <t>C</t>
         </is>
       </c>
       <c r="H60" s="14" t="inlineStr">
         <is>
-          <t>AT</t>
+          <t>C</t>
         </is>
       </c>
       <c r="I60" s="14" t="inlineStr">
         <is>
-          <t>AT</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J60" s="14" t="inlineStr">
         <is>
-          <t>AT</t>
+          <t>C</t>
         </is>
       </c>
       <c r="K60" s="15">
@@ -5232,7 +5256,11 @@
           <t>Désactiver les styles et vérifier l'ordre de lecture.</t>
         </is>
       </c>
-      <c r="M60" s="16" t="n"/>
+      <c r="M60" s="16" t="inlineStr">
+        <is>
+          <t>22/09/2026 — Sans styles, lecture linéaire logique : lien d'évitement, en-tête, navigation, contenu, pied de page ; pas de réordonnancement CSS porteur de sens.</t>
+        </is>
+      </c>
       <c r="N60" s="17" t="inlineStr">
         <is>
           <t>Critère 10.3</t>
@@ -5793,37 +5821,37 @@
       </c>
       <c r="D69" s="14" t="inlineStr">
         <is>
-          <t>AT</t>
+          <t>C</t>
         </is>
       </c>
       <c r="E69" s="14" t="inlineStr">
         <is>
-          <t>AT</t>
+          <t>C</t>
         </is>
       </c>
       <c r="F69" s="14" t="inlineStr">
         <is>
-          <t>AT</t>
+          <t>C</t>
         </is>
       </c>
       <c r="G69" s="14" t="inlineStr">
         <is>
-          <t>AT</t>
+          <t>C</t>
         </is>
       </c>
       <c r="H69" s="14" t="inlineStr">
         <is>
-          <t>AT</t>
+          <t>C</t>
         </is>
       </c>
       <c r="I69" s="14" t="inlineStr">
         <is>
-          <t>AT</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J69" s="14" t="inlineStr">
         <is>
-          <t>AT</t>
+          <t>C</t>
         </is>
       </c>
       <c r="K69" s="15">
@@ -5835,7 +5863,11 @@
           <t>Espacement WCAG 1.4.12 injecté : aucun débordement horizontal ; aucun texte rogné détecté sur les pages du site (hors décor). Plaquette : couverture à hauteur fixe signalée. Contrôle visuel à faire.</t>
         </is>
       </c>
-      <c r="M69" s="16" t="n"/>
+      <c r="M69" s="16" t="inlineStr">
+        <is>
+          <t>22/09/2026 — Espacement WCAG 1.4.12 appliqué (feuille CSSOM, la CSP bloquant un &lt;style&gt; injecté) à 1280 et 375 px : aucun texte rogné ni défilement horizontal. Plaquette HTML : feuilles à hauteur fixe qui rognaient le texte sur grand écran, corrigé (hauteur minimale A4 à l'écran). Menu mobile ouvert vérifié à 375×560.</t>
+        </is>
+      </c>
       <c r="N69" s="17" t="inlineStr">
         <is>
           <t>Critère 10.12</t>
@@ -8527,7 +8559,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F9"/>
+  <dimension ref="A1:F12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -8823,6 +8855,102 @@
       <c r="F9" s="12" t="inlineStr">
         <is>
           <t>Corrigé le 21/09/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="12" t="inlineStr">
+        <is>
+          <t>9.3</t>
+        </is>
+      </c>
+      <c r="B10" s="12" t="inlineStr">
+        <is>
+          <t>Accueil</t>
+        </is>
+      </c>
+      <c r="C10" s="12" t="inlineStr">
+        <is>
+          <t>Grille des 4 repères chiffrés : liste visuelle balisée en div.</t>
+        </is>
+      </c>
+      <c r="D10" s="12" t="inlineStr">
+        <is>
+          <t>Balisage ul/li (role="list" conservé pour VoiceOver).</t>
+        </is>
+      </c>
+      <c r="E10" s="12" t="inlineStr">
+        <is>
+          <t>Faible</t>
+        </is>
+      </c>
+      <c r="F10" s="12" t="inlineStr">
+        <is>
+          <t>Corrigé le 22/09/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="12" t="inlineStr">
+        <is>
+          <t>10.12</t>
+        </is>
+      </c>
+      <c r="B11" s="12" t="inlineStr">
+        <is>
+          <t>Plaquette (HTML)</t>
+        </is>
+      </c>
+      <c r="C11" s="12" t="inlineStr">
+        <is>
+          <t>Feuilles A4 à hauteur fixe (overflow: hidden) : texte rogné jusqu'à 84 px avec l'espacement WCAG sur grand écran.</t>
+        </is>
+      </c>
+      <c r="D11" s="12" t="inlineStr">
+        <is>
+          <t>À l'écran, hauteur minimale A4 au lieu d'une hauteur fixe ; impression et PDF inchangés.</t>
+        </is>
+      </c>
+      <c r="E11" s="12" t="inlineStr">
+        <is>
+          <t>Faible</t>
+        </is>
+      </c>
+      <c r="F11" s="12" t="inlineStr">
+        <is>
+          <t>Corrigé le 22/09/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="12" t="inlineStr">
+        <is>
+          <t>8.7</t>
+        </is>
+      </c>
+      <c r="B12" s="12" t="inlineStr">
+        <is>
+          <t>Accueil, À propos</t>
+        </is>
+      </c>
+      <c r="C12" s="12" t="inlineStr">
+        <is>
+          <t>Mots anglais non balisés : « Tagline », « Community Manager », « gaming » (2 alternatives d'images).</t>
+        </is>
+      </c>
+      <c r="D12" s="12" t="inlineStr">
+        <is>
+          <t>Francisés (choix d'Andy) : « Devise du projet », « Animateur de communauté », « événement de jeu vidéo », « borne d'arcade ».</t>
+        </is>
+      </c>
+      <c r="E12" s="12" t="inlineStr">
+        <is>
+          <t>Faible</t>
+        </is>
+      </c>
+      <c r="F12" s="12" t="inlineStr">
+        <is>
+          <t>Corrigé le 22/09/2026</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
a11y : tests RGAA manuels, trois corrections (#293)
- 9.3 : repères chiffrés de l'accueil balisés en ul/li
- 10.12 : feuilles de la plaquette HTML en hauteur minimale A4 à l'écran,
  le texte n'est plus rogné quand l'espacement augmente (impression et
  PDF inchangés)
- 8.7 : anglicismes francisés (Devise du projet, Animateur de
  communauté, alternatives d'images sans « gaming »)

Grille d'audit mise à jour : 8.2, 9.1, 3.1, 10.2, 10.3 conformes ;
restent les 5 critères à tester au lecteur d'écran.

Co-authored-by: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/audit-rgaa/grille-audit-rgaa-pxlc.xlsx
+++ b/docs/audit-rgaa/grille-audit-rgaa-pxlc.xlsx
@@ -555,7 +555,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Pré-remplie le 21/09/2026 à partir du build du site (tests automatisés jsdom, axe-core, Playwright, calculs de contraste) et de la lecture du code. Les 7 non-conformités relevées ont été corrigées le même jour (onglet « Corrections »).</t>
+          <t>Pré-remplie le 21/09/2026 à partir du build du site (tests automatisés jsdom, axe-core, Playwright, calculs de contraste) et de la lecture du code. Les 7 non-conformités relevées ont été corrigées le même jour (onglet « Corrections »). Mise à jour le 22/09/2026 : validateur W3C passé, tests 3.1, 8.7, 9.1, 9.3, 10.2, 10.3 et 10.12 faits (3 nouvelles corrections). Restent les tests au lecteur d'écran (NVDA).</t>
         </is>
       </c>
     </row>
@@ -2056,7 +2056,7 @@
       </c>
       <c r="G13" s="14" t="inlineStr">
         <is>
-          <t>AT</t>
+          <t>C</t>
         </is>
       </c>
       <c r="H13" s="14" t="inlineStr">
@@ -2083,7 +2083,11 @@
           <t>Lien actif du menu : couleur + barre + aria-current="page". Champs requis : astérisque + légende « Champs requis ». Contact : vérifier que la carte distingue la zone autrement que par la couleur (numéros).</t>
         </is>
       </c>
-      <c r="M13" s="16" t="n"/>
+      <c r="M13" s="16" t="inlineStr">
+        <is>
+          <t>22/09/2026 — Carte des communes en niveaux de gris : les 4 communes de la zone restent identifiables par leurs pastilles numérotées et la légende textuelle.</t>
+        </is>
+      </c>
       <c r="N13" s="17" t="inlineStr">
         <is>
           <t>Critère 3.1</t>
@@ -4185,37 +4189,37 @@
       </c>
       <c r="D45" s="14" t="inlineStr">
         <is>
-          <t>AT</t>
+          <t>C</t>
         </is>
       </c>
       <c r="E45" s="14" t="inlineStr">
         <is>
-          <t>AT</t>
+          <t>C</t>
         </is>
       </c>
       <c r="F45" s="14" t="inlineStr">
         <is>
-          <t>AT</t>
+          <t>C</t>
         </is>
       </c>
       <c r="G45" s="14" t="inlineStr">
         <is>
-          <t>AT</t>
+          <t>C</t>
         </is>
       </c>
       <c r="H45" s="14" t="inlineStr">
         <is>
-          <t>AT</t>
+          <t>C</t>
         </is>
       </c>
       <c r="I45" s="14" t="inlineStr">
         <is>
-          <t>AT</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J45" s="14" t="inlineStr">
         <is>
-          <t>AT</t>
+          <t>C</t>
         </is>
       </c>
       <c r="K45" s="15">
@@ -4227,7 +4231,11 @@
           <t>Identifiant dupliqué de Projets corrigé le 21/09/2026 (carte renommée « projet-jouons-ensemble ») ; plus aucun id en double sur l'échantillon. Reste à passer le validateur W3C sur chaque page.</t>
         </is>
       </c>
-      <c r="M45" s="16" t="n"/>
+      <c r="M45" s="16" t="inlineStr">
+        <is>
+          <t>22/09/2026 — Nu Html Checker (validator.w3.org, vnu 26.9.16) sur les 7 pages : 0 erreur. Avertissements « info » seulement : role="list" voulu (VoiceOver), alerte CSP des &lt;style&gt; inline = faux positif (hashes présents dans style-src). aria-required redondant retiré (PR #292).</t>
+        </is>
+      </c>
       <c r="N45" s="17" t="inlineStr">
         <is>
           <t>Critère 8.2</t>
@@ -4520,37 +4528,37 @@
       </c>
       <c r="D50" s="14" t="inlineStr">
         <is>
-          <t>AT</t>
+          <t>C</t>
         </is>
       </c>
       <c r="E50" s="14" t="inlineStr">
         <is>
-          <t>AT</t>
+          <t>C</t>
         </is>
       </c>
       <c r="F50" s="14" t="inlineStr">
         <is>
-          <t>AT</t>
+          <t>C</t>
         </is>
       </c>
       <c r="G50" s="14" t="inlineStr">
         <is>
-          <t>AT</t>
+          <t>C</t>
         </is>
       </c>
       <c r="H50" s="14" t="inlineStr">
         <is>
-          <t>AT</t>
+          <t>C</t>
         </is>
       </c>
       <c r="I50" s="14" t="inlineStr">
         <is>
-          <t>AT</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J50" s="14" t="inlineStr">
         <is>
-          <t>AT</t>
+          <t>C</t>
         </is>
       </c>
       <c r="K50" s="15">
@@ -4562,7 +4570,11 @@
           <t>Aucun changement de langue déclaré. Vérifier les mots anglais non passés dans l'usage (« gaming », « Duo gaming ») ; les noms propres (Destreland Gaming Cup) sont exemptés.</t>
         </is>
       </c>
-      <c r="M50" s="16" t="n"/>
+      <c r="M50" s="16" t="inlineStr">
+        <is>
+          <t>22/09/2026 — Relevé des mots étrangers : noms propres exemptés (Destreland Gaming Cup, Game Over Challenge, Atlantica Online, LinkedIn) ; esport, email, design dans l'usage. Francisés : « Tagline » → « Devise », « Community Manager » → « Animateur de communauté », « gaming » retiré de 2 alternatives d'images.</t>
+        </is>
+      </c>
       <c r="N50" s="17" t="inlineStr">
         <is>
           <t>Critère 8.7</t>
@@ -4788,7 +4800,7 @@
       </c>
       <c r="D54" s="14" t="inlineStr">
         <is>
-          <t>AT</t>
+          <t>C</t>
         </is>
       </c>
       <c r="E54" s="14" t="inlineStr">
@@ -4830,7 +4842,11 @@
           <t>Hiérarchie h1→h2→h3 cohérente. Accueil : « Quelques repères » et « Partenaires de confiance » ont l'apparence d'intitulés de section sans être des titres hx — à arbitrer.</t>
         </is>
       </c>
-      <c r="M54" s="16" t="n"/>
+      <c r="M54" s="16" t="inlineStr">
+        <is>
+          <t>22/09/2026 — « Quelques repères » balisé en h2 (PR #288) ; « Partenaires de confiance » est le libellé de la section PartnerStrip, nommée par aria-label.</t>
+        </is>
+      </c>
       <c r="N54" s="17" t="inlineStr">
         <is>
           <t>Critère 9.1</t>
@@ -4922,7 +4938,7 @@
       </c>
       <c r="D56" s="14" t="inlineStr">
         <is>
-          <t>AT</t>
+          <t>C</t>
         </is>
       </c>
       <c r="E56" s="14" t="inlineStr">
@@ -4964,7 +4980,11 @@
           <t>Listes balisées (ul/ol/dl). Accueil : vérifier la grille des 4 repères chiffrés, visuellement une liste mais balisée en div.</t>
         </is>
       </c>
-      <c r="M56" s="16" t="n"/>
+      <c r="M56" s="16" t="inlineStr">
+        <is>
+          <t>22/09/2026 — Les 4 repères chiffrés de l'accueil passent de div en ul/li (liste non ordonnée).</t>
+        </is>
+      </c>
       <c r="N56" s="17" t="inlineStr">
         <is>
           <t>Critère 9.3</t>
@@ -5123,37 +5143,37 @@
       </c>
       <c r="D59" s="14" t="inlineStr">
         <is>
-          <t>AT</t>
+          <t>C</t>
         </is>
       </c>
       <c r="E59" s="14" t="inlineStr">
         <is>
-          <t>AT</t>
+          <t>C</t>
         </is>
       </c>
       <c r="F59" s="14" t="inlineStr">
         <is>
-          <t>AT</t>
+          <t>C</t>
         </is>
       </c>
       <c r="G59" s="14" t="inlineStr">
         <is>
-          <t>AT</t>
+          <t>C</t>
         </is>
       </c>
       <c r="H59" s="14" t="inlineStr">
         <is>
-          <t>AT</t>
+          <t>C</t>
         </is>
       </c>
       <c r="I59" s="14" t="inlineStr">
         <is>
-          <t>AT</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J59" s="14" t="inlineStr">
         <is>
-          <t>AT</t>
+          <t>C</t>
         </is>
       </c>
       <c r="K59" s="15">
@@ -5165,7 +5185,11 @@
           <t>Désactiver les styles et vérifier que rien de porteur d'information ne disparaît (flèches → et points corail sont décoratifs).</t>
         </is>
       </c>
-      <c r="M59" s="16" t="n"/>
+      <c r="M59" s="16" t="inlineStr">
+        <is>
+          <t>22/09/2026 — Feuilles de style désactivées sur les 7 pages : tout le texte porteur d'information reste présent (contenus CSS générés = flèches, point, séparateurs, +/− de FAQ, tous décoratifs).</t>
+        </is>
+      </c>
       <c r="N59" s="17" t="inlineStr">
         <is>
           <t>Critère 10.2</t>
@@ -5190,37 +5214,37 @@
       </c>
       <c r="D60" s="14" t="inlineStr">
         <is>
-          <t>AT</t>
+          <t>C</t>
         </is>
       </c>
       <c r="E60" s="14" t="inlineStr">
         <is>
-          <t>AT</t>
+          <t>C</t>
         </is>
       </c>
       <c r="F60" s="14" t="inlineStr">
         <is>
-          <t>AT</t>
+          <t>C</t>
         </is>
       </c>
       <c r="G60" s="14" t="inlineStr">
         <is>
-          <t>AT</t>
+          <t>C</t>
         </is>
       </c>
       <c r="H60" s="14" t="inlineStr">
         <is>
-          <t>AT</t>
+          <t>C</t>
         </is>
       </c>
       <c r="I60" s="14" t="inlineStr">
         <is>
-          <t>AT</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J60" s="14" t="inlineStr">
         <is>
-          <t>AT</t>
+          <t>C</t>
         </is>
       </c>
       <c r="K60" s="15">
@@ -5232,7 +5256,11 @@
           <t>Désactiver les styles et vérifier l'ordre de lecture.</t>
         </is>
       </c>
-      <c r="M60" s="16" t="n"/>
+      <c r="M60" s="16" t="inlineStr">
+        <is>
+          <t>22/09/2026 — Sans styles, lecture linéaire logique : lien d'évitement, en-tête, navigation, contenu, pied de page ; pas de réordonnancement CSS porteur de sens.</t>
+        </is>
+      </c>
       <c r="N60" s="17" t="inlineStr">
         <is>
           <t>Critère 10.3</t>
@@ -5793,37 +5821,37 @@
       </c>
       <c r="D69" s="14" t="inlineStr">
         <is>
-          <t>AT</t>
+          <t>C</t>
         </is>
       </c>
       <c r="E69" s="14" t="inlineStr">
         <is>
-          <t>AT</t>
+          <t>C</t>
         </is>
       </c>
       <c r="F69" s="14" t="inlineStr">
         <is>
-          <t>AT</t>
+          <t>C</t>
         </is>
       </c>
       <c r="G69" s="14" t="inlineStr">
         <is>
-          <t>AT</t>
+          <t>C</t>
         </is>
       </c>
       <c r="H69" s="14" t="inlineStr">
         <is>
-          <t>AT</t>
+          <t>C</t>
         </is>
       </c>
       <c r="I69" s="14" t="inlineStr">
         <is>
-          <t>AT</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J69" s="14" t="inlineStr">
         <is>
-          <t>AT</t>
+          <t>C</t>
         </is>
       </c>
       <c r="K69" s="15">
@@ -5835,7 +5863,11 @@
           <t>Espacement WCAG 1.4.12 injecté : aucun débordement horizontal ; aucun texte rogné détecté sur les pages du site (hors décor). Plaquette : couverture à hauteur fixe signalée. Contrôle visuel à faire.</t>
         </is>
       </c>
-      <c r="M69" s="16" t="n"/>
+      <c r="M69" s="16" t="inlineStr">
+        <is>
+          <t>22/09/2026 — Espacement WCAG 1.4.12 appliqué (feuille CSSOM, la CSP bloquant un &lt;style&gt; injecté) à 1280 et 375 px : aucun texte rogné ni défilement horizontal. Plaquette HTML : feuilles à hauteur fixe qui rognaient le texte sur grand écran, corrigé (hauteur minimale A4 à l'écran). Menu mobile ouvert vérifié à 375×560.</t>
+        </is>
+      </c>
       <c r="N69" s="17" t="inlineStr">
         <is>
           <t>Critère 10.12</t>
@@ -8527,7 +8559,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F9"/>
+  <dimension ref="A1:F12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -8823,6 +8855,102 @@
       <c r="F9" s="12" t="inlineStr">
         <is>
           <t>Corrigé le 21/09/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="12" t="inlineStr">
+        <is>
+          <t>9.3</t>
+        </is>
+      </c>
+      <c r="B10" s="12" t="inlineStr">
+        <is>
+          <t>Accueil</t>
+        </is>
+      </c>
+      <c r="C10" s="12" t="inlineStr">
+        <is>
+          <t>Grille des 4 repères chiffrés : liste visuelle balisée en div.</t>
+        </is>
+      </c>
+      <c r="D10" s="12" t="inlineStr">
+        <is>
+          <t>Balisage ul/li (role="list" conservé pour VoiceOver).</t>
+        </is>
+      </c>
+      <c r="E10" s="12" t="inlineStr">
+        <is>
+          <t>Faible</t>
+        </is>
+      </c>
+      <c r="F10" s="12" t="inlineStr">
+        <is>
+          <t>Corrigé le 22/09/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="12" t="inlineStr">
+        <is>
+          <t>10.12</t>
+        </is>
+      </c>
+      <c r="B11" s="12" t="inlineStr">
+        <is>
+          <t>Plaquette (HTML)</t>
+        </is>
+      </c>
+      <c r="C11" s="12" t="inlineStr">
+        <is>
+          <t>Feuilles A4 à hauteur fixe (overflow: hidden) : texte rogné jusqu'à 84 px avec l'espacement WCAG sur grand écran.</t>
+        </is>
+      </c>
+      <c r="D11" s="12" t="inlineStr">
+        <is>
+          <t>À l'écran, hauteur minimale A4 au lieu d'une hauteur fixe ; impression et PDF inchangés.</t>
+        </is>
+      </c>
+      <c r="E11" s="12" t="inlineStr">
+        <is>
+          <t>Faible</t>
+        </is>
+      </c>
+      <c r="F11" s="12" t="inlineStr">
+        <is>
+          <t>Corrigé le 22/09/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="12" t="inlineStr">
+        <is>
+          <t>8.7</t>
+        </is>
+      </c>
+      <c r="B12" s="12" t="inlineStr">
+        <is>
+          <t>Accueil, À propos</t>
+        </is>
+      </c>
+      <c r="C12" s="12" t="inlineStr">
+        <is>
+          <t>Mots anglais non balisés : « Tagline », « Community Manager », « gaming » (2 alternatives d'images).</t>
+        </is>
+      </c>
+      <c r="D12" s="12" t="inlineStr">
+        <is>
+          <t>Francisés (choix d'Andy) : « Devise du projet », « Animateur de communauté », « événement de jeu vidéo », « borne d'arcade ».</t>
+        </is>
+      </c>
+      <c r="E12" s="12" t="inlineStr">
+        <is>
+          <t>Faible</t>
+        </is>
+      </c>
+      <c r="F12" s="12" t="inlineStr">
+        <is>
+          <t>Corrigé le 22/09/2026</t>
         </is>
       </c>
     </row>

</xml_diff>